<commit_message>
A13b: Cox decomposition restricted to patients at risk; Fig 1D/3B/4 updates; provenance-filtered label wording; SI (S10 A13b sheet, S1 Text history); README
</commit_message>
<xml_diff>
--- a/manuscript_v5/SI/S10_Table.xlsx
+++ b/manuscript_v5/SI/S10_Table.xlsx
@@ -11,9 +11,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A13_os_decomposition" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A13_clinical_only_auc" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A13_redaction" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A3_cox_hr" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A3_cox_summary" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A3_cox_ph" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A13b_decomposition" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A3_cox_hr" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A3_cox_summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A3_cox_ph" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,7 +455,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>S10 Table. Exploratory analyses (A13, added after the main results were known): decomposition of overall survival into the platinum-free interval and survival after progression; clinical-only models; exclusion of TCGA-CDR redacted records. Also the pre-specified Cox models of the TCGA-CDR progression-free interval (A3, R survival).</t>
+          <t>S10 Table. Exploratory analyses (A13, A13b; added after the main results were known): decomposition of overall survival into the platinum-free interval (A13b: patients at risk at the end of platinum; the earlier A13 model, which set intervals below 1 day to 1 day, as a sensitivity analysis) and survival after progression; clinical-only models; exclusion of TCGA-CDR redacted records. Also the pre-specified Cox models of the TCGA-CDR progression-free interval (A3, R survival).</t>
         </is>
       </c>
     </row>
@@ -466,7 +467,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>A13: label_validity/outputs/a13_os_decomposition_cox.csv, label_validity/outputs/a13_clinical_only_auc.csv, label_validity/outputs/a13_redaction.csv</t>
+          <t>A13b (reported decomposition: platinum-free interval in the 408 patients at risk at the end of platinum; column analysis = at_risk / clipped_as_A13 sensitivity / unchanged): label_validity/outputs/a13b_decomposition_cox.csv</t>
         </is>
       </c>
     </row>
@@ -477,6 +478,18 @@
         </is>
       </c>
       <c r="B4" t="inlineStr">
+        <is>
+          <t>A13: label_validity/outputs/a13_os_decomposition_cox.csv, label_validity/outputs/a13_clinical_only_auc.csv, label_validity/outputs/a13_redaction.csv (A13 decomposition set intervals below 1 day to 1 day; superseded by A13b)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>source / note</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>A3 Cox: label_validity/outputs/a3_pfi_cox_hr.csv, label_validity/outputs/a3_pfi_cox_summary.csv, label_validity/outputs/a3_pfi_cox_ph.csv (cohort of 432 patients with any 'platin' agent; includes one oxaliplatin-only patient not in the 489)</t>
         </is>
@@ -1423,36 +1436,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>analysis</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>term</t>
+          <t>covariate</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>outcome</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>HR_lo</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>HR_hi</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>lo</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>p</t>
         </is>
@@ -1461,169 +1489,736 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>pfi_baseline_full</t>
+          <t>at_risk</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>log_tmb</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>0.896835825133224</v>
+          <t>age10</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PFI_from_platinum</t>
+        </is>
       </c>
       <c r="D2" t="n">
-        <v>0.76153881095512</v>
+        <v>408</v>
       </c>
       <c r="E2" t="n">
-        <v>1.05617006733199</v>
+        <v>316</v>
       </c>
       <c r="F2" t="n">
-        <v>0.191899392929725</v>
+        <v>1.087143081797776</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.9843368083278564</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.200686665683554</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.09925280267651319</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>pfi_baseline_full</t>
+          <t>clipped_as_A13</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aneu</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>1.0276073472705</v>
+          <t>age10</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PFI_from_platinum</t>
+        </is>
       </c>
       <c r="D3" t="n">
-        <v>1.01209692814653</v>
+        <v>436</v>
       </c>
       <c r="E3" t="n">
-        <v>1.04335546408399</v>
+        <v>328</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0004488708360428</v>
+        <v>1.081840077396254</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.981378152550286</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.192586109665574</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.1136626748745072</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>pfi_baseline_matched</t>
+          <t>unchanged</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>log_tmb</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>0.693012595774222</v>
+          <t>age10</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>survival_after_progression</t>
+        </is>
       </c>
       <c r="D4" t="n">
-        <v>0.518940002981244</v>
+        <v>331</v>
       </c>
       <c r="E4" t="n">
-        <v>0.925475883806714</v>
+        <v>237</v>
       </c>
       <c r="F4" t="n">
-        <v>0.012964976752954</v>
+        <v>1.258548520674536</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.11615025978159</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.419113927547723</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.0001742938592468</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>pfi_baseline_matched</t>
+          <t>at_risk</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>aneu</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>1.02848478873593</v>
+          <t>stage_iv</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PFI_from_platinum</t>
+        </is>
       </c>
       <c r="D5" t="n">
-        <v>1.00970474547555</v>
+        <v>407</v>
       </c>
       <c r="E5" t="n">
-        <v>1.04761413215207</v>
+        <v>315</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0028161342131732</v>
+        <v>1.289319236353506</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.9615633371492744</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.728793131983904</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.0894974885924876</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>pfi_brca_added</t>
+          <t>clipped_as_A13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>log_tmb</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0.761589909268892</v>
+          <t>stage_iv</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PFI_from_platinum</t>
+        </is>
       </c>
       <c r="D6" t="n">
-        <v>0.565066458329317</v>
+        <v>435</v>
       </c>
       <c r="E6" t="n">
-        <v>1.02646189903944</v>
+        <v>327</v>
       </c>
       <c r="F6" t="n">
-        <v>0.073702961987719</v>
+        <v>1.282501140992606</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.9615797609901848</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.710528074086749</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.09039207354013989</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>pfi_brca_added</t>
+          <t>unchanged</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>aneu</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>1.0260311640151</v>
+          <t>stage_iv</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>survival_after_progression</t>
+        </is>
       </c>
       <c r="D7" t="n">
-        <v>1.00731963639093</v>
+        <v>331</v>
       </c>
       <c r="E7" t="n">
-        <v>1.0450902687671</v>
+        <v>237</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0062078982662556</v>
+        <v>1.029348211728684</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.7412157485035611</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.429486277279157</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.8629334819934353</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>pfi_brca_added</t>
+          <t>at_risk</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BRCA_any_mutated</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0.498974823859485</v>
+          <t>residual_subopt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>PFI_from_platinum</t>
+        </is>
       </c>
       <c r="D8" t="n">
-        <v>0.286689702928274</v>
+        <v>322</v>
       </c>
       <c r="E8" t="n">
-        <v>0.868450705771927</v>
+        <v>261</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0139395608279276</v>
+        <v>1.075188792791683</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.820360008568779</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.409175152457368</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.5993950073972188</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>clipped_as_A13</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>residual_subopt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PFI_from_platinum</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>349</v>
+      </c>
+      <c r="E9" t="n">
+        <v>273</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.106505273537036</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.8507957126687654</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1.439069217362101</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.4503516852915932</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>unchanged</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>residual_subopt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>survival_after_progression</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>267</v>
+      </c>
+      <c r="E10" t="n">
+        <v>202</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1.4113518831148</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.031747778210372</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1.930621204173356</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.0311234876892053</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>at_risk</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>resid_any</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>PFI_from_platinum</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>322</v>
+      </c>
+      <c r="E11" t="n">
+        <v>261</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.640698444110172</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.206735802196474</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2.230721405303313</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.0015836973158879</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>clipped_as_A13</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>resid_any</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PFI_from_platinum</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>349</v>
+      </c>
+      <c r="E12" t="n">
+        <v>273</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.66765109161259</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.231260321061063</v>
+      </c>
+      <c r="H12" t="n">
+        <v>2.258710132849914</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.0009531934341207</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>unchanged</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>resid_any</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>survival_after_progression</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>267</v>
+      </c>
+      <c r="E13" t="n">
+        <v>202</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.660894679288078</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1.112427498798069</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2.479776110054782</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.0131027125946976</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>at_risk</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>brca_carrier</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>PFI_from_platinum</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>236</v>
+      </c>
+      <c r="E14" t="n">
+        <v>195</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.5461941514846266</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.3767589528542565</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.7918273709381896</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.001413716875106</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>clipped_as_A13</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>brca_carrier</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PFI_from_platinum</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>247</v>
+      </c>
+      <c r="E15" t="n">
+        <v>202</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.5489529183809438</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.3807426919394934</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.7914775857256501</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.0013151522366995</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>unchanged</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>brca_carrier</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>survival_after_progression</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>201</v>
+      </c>
+      <c r="E16" t="n">
+        <v>152</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.6807707171227614</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.4361956972274942</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1.062479002515541</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.0904334224452981</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>at_risk</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ccne1_amp</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>PFI_from_platinum</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>356</v>
+      </c>
+      <c r="E17" t="n">
+        <v>285</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1.578740971884279</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1.191851197906119</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2.091219995151144</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.0014545527294249</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>clipped_as_A13</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ccne1_amp</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>PFI_from_platinum</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>384</v>
+      </c>
+      <c r="E18" t="n">
+        <v>297</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.564151602691813</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1.188193452769412</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2.059067259208475</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.0014260281395451</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>unchanged</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ccne1_amp</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>survival_after_progression</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>294</v>
+      </c>
+      <c r="E19" t="n">
+        <v>218</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1.184199469801454</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.8620691446280485</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1.626700587785332</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.2966180079970801</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>at_risk</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>aneuploidy_sd</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>PFI_from_platinum</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>390</v>
+      </c>
+      <c r="E20" t="n">
+        <v>301</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1.23139666568302</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.098015733549925</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1.38097998227483</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.0003729458255508</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>clipped_as_A13</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>aneuploidy_sd</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>PFI_from_platinum</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>418</v>
+      </c>
+      <c r="E21" t="n">
+        <v>313</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1.202874837973244</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1.07470806868293</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1.346326428536414</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.0013119462066407</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>unchanged</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>aneuploidy_sd</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>survival_after_progression</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>317</v>
+      </c>
+      <c r="E22" t="n">
+        <v>225</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1.026195738881403</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.8969729728421968</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1.174035033811008</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.7064936339632832</v>
       </c>
     </row>
   </sheetData>
@@ -1637,7 +2232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1648,22 +2243,27 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>term</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>events</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>c_index</t>
+          <t>HR_lo</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>c_index_se</t>
+          <t>HR_hi</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>p</t>
         </is>
       </c>
     </row>
@@ -1673,55 +2273,166 @@
           <t>pfi_baseline_full</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>432</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>log_tmb</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>317</v>
+        <v>0.896835825133224</v>
       </c>
       <c r="D2" t="n">
-        <v>0.559619383158138</v>
+        <v>0.76153881095512</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0191188015969111</v>
+        <v>1.05617006733199</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.191899392929725</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>pfi_baseline_matched</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>335</v>
+          <t>pfi_baseline_full</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>aneu</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>236</v>
+        <v>1.0276073472705</v>
       </c>
       <c r="D3" t="n">
-        <v>0.561980396181874</v>
+        <v>1.01209692814653</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0198849591811109</v>
+        <v>1.04335546408399</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0004488708360428</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>pfi_baseline_matched</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>log_tmb</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.693012595774222</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.518940002981244</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.925475883806714</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.012964976752954</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>pfi_baseline_matched</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>aneu</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1.02848478873593</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.00970474547555</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.04761413215207</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.0028161342131732</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>pfi_brca_added</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>335</v>
-      </c>
-      <c r="C4" t="n">
-        <v>236</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.573693934106538</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.0203739278625368</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>log_tmb</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.761589909268892</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.565066458329317</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.02646189903944</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.073702961987719</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>pfi_brca_added</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>aneu</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1.0260311640151</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.00731963639093</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.0450902687671</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.0062078982662556</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>pfi_brca_added</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BRCA_any_mutated</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.498974823859485</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.286689702928274</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.868450705771927</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.0139395608279276</v>
       </c>
     </row>
   </sheetData>
@@ -1735,6 +2446,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>c_index</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>c_index_se</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>pfi_baseline_full</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>432</v>
+      </c>
+      <c r="C2" t="n">
+        <v>317</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.559619383158138</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.0191188015969111</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>pfi_baseline_matched</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>335</v>
+      </c>
+      <c r="C3" t="n">
+        <v>236</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.561980396181874</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0198849591811109</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>pfi_brca_added</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>335</v>
+      </c>
+      <c r="C4" t="n">
+        <v>236</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.573693934106538</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0203739278625368</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
A18 anchor sensitivity, A19 IPCW, A20 documentation checks; SI and README updated
</commit_message>
<xml_diff>
--- a/manuscript_v5/SI/S10_Table.xlsx
+++ b/manuscript_v5/SI/S10_Table.xlsx
@@ -12,9 +12,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A13_clinical_only_auc" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A13_redaction" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A13b_decomposition" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A3_cox_hr" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A3_cox_summary" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A3_cox_ph" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A20_cox_checks" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A3_cox_hr" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A3_cox_summary" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A3_cox_ph" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2232,207 +2233,402 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>outcome</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>term</t>
+          <t>covariate</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>HR_lo</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>HR_hi</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>p</t>
+          <t>ph_test_p</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>quadratic_term_p</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>pfi_baseline_full</t>
+          <t>PFI_from_platinum</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>log_tmb</t>
+          <t>age10</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.896835825133224</v>
+        <v>408</v>
       </c>
       <c r="D2" t="n">
-        <v>0.76153881095512</v>
+        <v>316</v>
       </c>
       <c r="E2" t="n">
-        <v>1.05617006733199</v>
+        <v>1.087143081797776</v>
       </c>
       <c r="F2" t="n">
-        <v>0.191899392929725</v>
+        <v>0.0397132019019213</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.6762173906827009</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>pfi_baseline_full</t>
+          <t>PFI_from_platinum</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aneu</t>
+          <t>stage_iv</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.0276073472705</v>
+        <v>407</v>
       </c>
       <c r="D3" t="n">
-        <v>1.01209692814653</v>
+        <v>315</v>
       </c>
       <c r="E3" t="n">
-        <v>1.04335546408399</v>
+        <v>1.289319236353506</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0004488708360428</v>
-      </c>
+        <v>0.5701510295594943</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>pfi_baseline_matched</t>
+          <t>PFI_from_platinum</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>log_tmb</t>
+          <t>residual_subopt</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.693012595774222</v>
+        <v>322</v>
       </c>
       <c r="D4" t="n">
-        <v>0.518940002981244</v>
+        <v>261</v>
       </c>
       <c r="E4" t="n">
-        <v>0.925475883806714</v>
+        <v>1.075188792791683</v>
       </c>
       <c r="F4" t="n">
-        <v>0.012964976752954</v>
-      </c>
+        <v>0.9155302077472248</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>pfi_baseline_matched</t>
+          <t>PFI_from_platinum</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>aneu</t>
+          <t>resid_any</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.02848478873593</v>
+        <v>322</v>
       </c>
       <c r="D5" t="n">
-        <v>1.00970474547555</v>
+        <v>261</v>
       </c>
       <c r="E5" t="n">
-        <v>1.04761413215207</v>
+        <v>1.640698444110172</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0028161342131732</v>
-      </c>
+        <v>0.2289130213870076</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>pfi_brca_added</t>
+          <t>PFI_from_platinum</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>log_tmb</t>
+          <t>brca_carrier</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.761589909268892</v>
+        <v>236</v>
       </c>
       <c r="D6" t="n">
-        <v>0.565066458329317</v>
+        <v>195</v>
       </c>
       <c r="E6" t="n">
-        <v>1.02646189903944</v>
+        <v>0.5461941514846266</v>
       </c>
       <c r="F6" t="n">
-        <v>0.073702961987719</v>
-      </c>
+        <v>0.997836660147612</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>pfi_brca_added</t>
+          <t>PFI_from_platinum</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>aneu</t>
+          <t>ccne1_amp</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.0260311640151</v>
+        <v>356</v>
       </c>
       <c r="D7" t="n">
-        <v>1.00731963639093</v>
+        <v>285</v>
       </c>
       <c r="E7" t="n">
-        <v>1.0450902687671</v>
+        <v>1.578740971884279</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0062078982662556</v>
-      </c>
+        <v>0.4814942232111823</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>pfi_brca_added</t>
+          <t>PFI_from_platinum</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BRCA_any_mutated</t>
+          <t>aneuploidy_sd</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.498974823859485</v>
+        <v>390</v>
       </c>
       <c r="D8" t="n">
-        <v>0.286689702928274</v>
+        <v>301</v>
       </c>
       <c r="E8" t="n">
-        <v>0.868450705771927</v>
+        <v>1.23139666568302</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0139395608279276</v>
+        <v>0.2666279285008983</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.7128825433131536</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>survival_after_progression</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>age10</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>331</v>
+      </c>
+      <c r="D9" t="n">
+        <v>237</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1.258548520674536</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.15503652268171</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.5668727484143186</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>survival_after_progression</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>stage_iv</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>331</v>
+      </c>
+      <c r="D10" t="n">
+        <v>237</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1.029348211728684</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.7600432087631479</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>survival_after_progression</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>residual_subopt</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>267</v>
+      </c>
+      <c r="D11" t="n">
+        <v>202</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.4113518831148</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.3422257578761755</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>survival_after_progression</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>resid_any</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>267</v>
+      </c>
+      <c r="D12" t="n">
+        <v>202</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.660894679288078</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.7361568213159317</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>survival_after_progression</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>brca_carrier</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>201</v>
+      </c>
+      <c r="D13" t="n">
+        <v>152</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.6807707171227614</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.3087962810829948</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>survival_after_progression</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ccne1_amp</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>294</v>
+      </c>
+      <c r="D14" t="n">
+        <v>218</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1.184199469801454</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.1676051866023159</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>survival_after_progression</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>aneuploidy_sd</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>317</v>
+      </c>
+      <c r="D15" t="n">
+        <v>225</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.026195738881403</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.0217350910785281</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.2810809303312978</v>
       </c>
     </row>
   </sheetData>
@@ -2446,7 +2642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2457,22 +2653,27 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>term</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>events</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>c_index</t>
+          <t>HR_lo</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>c_index_se</t>
+          <t>HR_hi</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>p</t>
         </is>
       </c>
     </row>
@@ -2482,55 +2683,166 @@
           <t>pfi_baseline_full</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>432</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>log_tmb</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>317</v>
+        <v>0.896835825133224</v>
       </c>
       <c r="D2" t="n">
-        <v>0.559619383158138</v>
+        <v>0.76153881095512</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0191188015969111</v>
+        <v>1.05617006733199</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.191899392929725</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>pfi_baseline_matched</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>335</v>
+          <t>pfi_baseline_full</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>aneu</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>236</v>
+        <v>1.0276073472705</v>
       </c>
       <c r="D3" t="n">
-        <v>0.561980396181874</v>
+        <v>1.01209692814653</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0198849591811109</v>
+        <v>1.04335546408399</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0004488708360428</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>pfi_baseline_matched</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>log_tmb</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.693012595774222</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.518940002981244</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.925475883806714</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.012964976752954</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>pfi_baseline_matched</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>aneu</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1.02848478873593</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.00970474547555</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.04761413215207</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.0028161342131732</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>pfi_brca_added</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>335</v>
-      </c>
-      <c r="C4" t="n">
-        <v>236</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.573693934106538</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.0203739278625368</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>log_tmb</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.761589909268892</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.565066458329317</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.02646189903944</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.073702961987719</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>pfi_brca_added</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>aneu</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1.0260311640151</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.00731963639093</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.0450902687671</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.0062078982662556</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>pfi_brca_added</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BRCA_any_mutated</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.498974823859485</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.286689702928274</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.868450705771927</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.0139395608279276</v>
       </c>
     </row>
   </sheetData>
@@ -2544,6 +2856,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>c_index</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>c_index_se</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>pfi_baseline_full</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>432</v>
+      </c>
+      <c r="C2" t="n">
+        <v>317</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.559619383158138</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.0191188015969111</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>pfi_baseline_matched</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>335</v>
+      </c>
+      <c r="C3" t="n">
+        <v>236</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.561980396181874</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0198849591811109</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>pfi_brca_added</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>335</v>
+      </c>
+      <c r="C4" t="n">
+        <v>236</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.573693934106538</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0203739278625368</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
A21 event-type sensitivity; A22 full-pipeline bootstrap; Fig 3B; SI, README
</commit_message>
<xml_diff>
--- a/manuscript_v5/SI/S10_Table.xlsx
+++ b/manuscript_v5/SI/S10_Table.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,6 +491,18 @@
         </is>
       </c>
       <c r="B5" t="inlineStr">
+        <is>
+          <t>A20: label_validity/outputs/a20_cox_checks.csv (proportional-hazards tests and quadratic-term checks for the A13b models)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>source / note</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>A3 Cox: label_validity/outputs/a3_pfi_cox_hr.csv, label_validity/outputs/a3_pfi_cox_summary.csv, label_validity/outputs/a3_pfi_cox_ph.csv (cohort of 432 patients with any 'platin' agent; includes one oxaliplatin-only patient not in the 489)</t>
         </is>

</xml_diff>